<commit_message>
Add hub topic model (T-01) + in-memory bus (T-02); wire Dashboard/Registry to real APIs (T-07)
Hub Engine (Sprint 1):
- T-01: hub/topic.ts canonical source.entity.event topic model (validate/parse/
  build + centralized topicMatches); topic validation + idempotency-key-derived
  messageId in createEnvelope; router uses shared matcher; hardened SP-source slug.
- T-02: in-memory IntegrationBus (direction A) - SubscriptionRegistry (org-scoped
  findMatching), BoundedQueue (FIFO async channel w/ backpressure), InMemoryBus
  (publish->queue->router fan-out, checksum validation, transform hook).

Frontend (T-07):
- Wire Dashboard + Registry to /api/connected via shared integrationMap.js; live
  KPIs/tiles/charts with sample-data fallback.

Tests: 76 hub tests pass (+34 new across topic/envelope/bus suites). Plan v3 updated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Synapse_Project_Plan_v3.xlsx
+++ b/Synapse_Project_Plan_v3.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Decisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Milestones" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sprint Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Risks &amp; Decisions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -655,7 +655,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -1114,11 +1114,11 @@
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H2" s="16" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="I2" s="17" t="n">
         <v>46160</v>
@@ -1126,14 +1126,16 @@
       <c r="J2" s="17" t="n">
         <v>46171</v>
       </c>
-      <c r="K2" s="17" t="n"/>
+      <c r="K2" s="17" t="n">
+        <v>46176</v>
+      </c>
       <c r="L2" s="14">
         <f>IF(K2="","",IF(K2&lt;=J2,"On-Time","Late"))</f>
         <v/>
       </c>
       <c r="M2" s="15" t="inlineStr">
         <is>
-          <t>Team began 18 May. Immutable envelope, idempotency key.</t>
+          <t>COMPLETE (T-01) — immutable envelope + SHA-256 checksum existed; added hub/topic.ts (canonical source.entity.event, validate/parse/build, centralized topicMatches), topic validation + idempotency-key-derived messageId in createEnvelope, router refactor. 59 hub tests pass.</t>
         </is>
       </c>
     </row>
@@ -1386,11 +1388,11 @@
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H7" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" s="17" t="n">
         <v>46160</v>
@@ -1398,14 +1400,16 @@
       <c r="J7" s="17" t="n">
         <v>46171</v>
       </c>
-      <c r="K7" s="17" t="n"/>
+      <c r="K7" s="17" t="n">
+        <v>46175</v>
+      </c>
       <c r="L7" s="14">
         <f>IF(K7="","",IF(K7&lt;=J7,"On-Time","Late"))</f>
         <v/>
       </c>
       <c r="M7" s="15" t="inlineStr">
         <is>
-          <t>Reuse SP source + type mapper.</t>
+          <t>COMPLETE (T-06) — SqlServerWriter smartUpsert + sys.columns introspect + hub MSSQL endpoints + wizard wiring. Tested.</t>
         </is>
       </c>
     </row>
@@ -1440,11 +1444,11 @@
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H8" s="16" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="I8" s="17" t="n">
         <v>46160</v>
@@ -1459,7 +1463,7 @@
       </c>
       <c r="M8" s="15" t="inlineStr">
         <is>
-          <t>First real-data screens.</t>
+          <t>T-07 code-complete: integrationMap.js shared mapper, live KPIs/tiles/charts off /api/connected, sample fallback, 0 diagnostics. Pending browser verify for M1.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
snapshot before dead-code cleanup
Checkpoint of ~12 days of uncommitted work (QC-safe features, entity-join,
file-share, web-scraping, multi-target fan-out, Clients build + removal) so the
dead-code cleanup that follows is revertable file-by-file.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Synapse_Project_Plan_v3.xlsx
+++ b/Synapse_Project_Plan_v3.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Milestones" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sprint Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Risks &amp; Decisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Decisions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1784,11 +1784,11 @@
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H14" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" s="17" t="n">
         <v>46188</v>
@@ -1796,14 +1796,16 @@
       <c r="J14" s="17" t="n">
         <v>46199</v>
       </c>
-      <c r="K14" s="17" t="n"/>
+      <c r="K14" s="17" t="n">
+        <v>46192</v>
+      </c>
       <c r="L14" s="14">
         <f>IF(K14="","",IF(K14&lt;=J14,"On-Time","Late"))</f>
         <v/>
       </c>
       <c r="M14" s="15" t="inlineStr">
         <is>
-          <t>NEW. Subscription -&gt; enforced level of access.</t>
+          <t>COMPLETE (2026-06-19 Admin/Auth build) - real JWT login (jose+bcrypt), actor-seam token verification + AUTH_REQUIRED prod gate (enforcement), users+roles + RBAC nav, admin UI. Dev login admin@synapse.local.</t>
         </is>
       </c>
     </row>
@@ -2004,11 +2006,11 @@
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" s="17" t="n">
         <v>46188</v>
@@ -2016,14 +2018,16 @@
       <c r="J18" s="17" t="n">
         <v>46199</v>
       </c>
-      <c r="K18" s="17" t="n"/>
+      <c r="K18" s="17" t="n">
+        <v>46192</v>
+      </c>
       <c r="L18" s="14">
         <f>IF(K18="","",IF(K18&lt;=J18,"On-Time","Late"))</f>
         <v/>
       </c>
       <c r="M18" s="15" t="inlineStr">
         <is>
-          <t>Append-only, before/after diff.</t>
+          <t>COMPLETE (2026-06-19 Admin/Auth build) - audit-log write path + Audit Viewer UI; actor/action recorded across privileged routes.</t>
         </is>
       </c>
     </row>
@@ -2278,11 +2282,11 @@
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H23" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" s="17" t="n">
         <v>46202</v>
@@ -2290,14 +2294,16 @@
       <c r="J23" s="17" t="n">
         <v>46213</v>
       </c>
-      <c r="K23" s="17" t="n"/>
+      <c r="K23" s="17" t="n">
+        <v>46192</v>
+      </c>
       <c r="L23" s="14">
         <f>IF(K23="","",IF(K23&lt;=J23,"On-Time","Late"))</f>
         <v/>
       </c>
       <c r="M23" s="15" t="inlineStr">
         <is>
-          <t>Next-run preview.</t>
+          <t>COMPLETE - SchedulerService.initScheduler wired into hub boot (BullMQ repeatable jobs via upsertJobScheduler); per-connection schedule managed from the Connected page. Cron-builder UI is minimal.</t>
         </is>
       </c>
     </row>
@@ -2332,11 +2338,11 @@
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H24" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" s="17" t="n">
         <v>46202</v>
@@ -2344,14 +2350,16 @@
       <c r="J24" s="17" t="n">
         <v>46213</v>
       </c>
-      <c r="K24" s="17" t="n"/>
+      <c r="K24" s="17" t="n">
+        <v>46192</v>
+      </c>
       <c r="L24" s="14">
         <f>IF(K24="","",IF(K24&lt;=J24,"On-Time","Late"))</f>
         <v/>
       </c>
       <c r="M24" s="15" t="inlineStr">
         <is>
-          <t>Existing engine regression.</t>
+          <t>COMPLETE - Jira-&gt;SharePoint moved onto the IntegrationBus (bus-egress cutover) + push-reliability hardening / connection de-dup; delivered via the SharePoint destination with idempotency, retry/backoff and DLQ.</t>
         </is>
       </c>
     </row>

</xml_diff>